<commit_message>
IP & Licensing: impute office revenue at SKU list price
Office/external bookings show £0 in the DMN online system because
payment settles at the venue till. To give a complete picture of
Borough 2025 revenue, impute office revenue as qty × SKU list price.

- Office imputed total: £61,629 (4,512 tickets at list)
- Combined Borough 2025: £272,793 (online £211,164 + office £61,629)

- data.js: office SKU revenue populated per SKU; monthly officeRev
  filled; grand totals include totalRev £272,792.70
- IPLicensing.jsx: office table renders revenue (no longer greyed),
  stat cards show online actual + office imputed + combined total,
  monthly chart switched to revenue view
- xlsx: Office sheet column labelled "imputed at list price", Monthly
  sheet gains a Total Revenue column, README updated

Holding Co model still scoped to online-only revenue per earlier
decision — office/till sales bypass Holding Co entirely.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/ip_licensing_2025.xlsx
+++ b/workbook/ip_licensing_2025.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IP &amp; LICENSING — BOROUGH 2025 (split by channel)</t>
+          <t>IP &amp; LICENSING — BOROUGH 2025 (split by channel, all revenue coded in)</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: 'ALL DMN 2025 transactions ALL SITES.xlsx' — filtered to Borough venue only, split by Status.</t>
+          <t>Source: 'ALL DMN 2025 transactions ALL SITES.xlsx' — filtered to Borough venue only, split by Status column.</t>
         </is>
       </c>
     </row>
@@ -524,28 +524,28 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>KEY FINDING:</t>
+          <t>CHANNEL SPLIT:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • ONLINE (Status = complete):  15,188 tickets  £ 211,163.70   ← revenue through online system</t>
+          <t xml:space="preserve">  • ONLINE (Status = complete):  15,188 tickets  £ 211,163.70  ← actual portal revenue</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • OFFICE (Status = external):    4,512 tickets  £       0.00   ← settled at venue till (£0 online revenue)</t>
+          <t xml:space="preserve">  • OFFICE (Status = external):    4,512 tickets  £  61,629.00  ← IMPUTED at SKU list price (qty × price)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Online = 77.1% of ticket volume but 100% of revenue captured by the online system.</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • COMBINED 2025 Borough rev:    19,700 tickets  £ 272,792.70</t>
         </is>
       </c>
     </row>
@@ -555,28 +555,28 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>UNDER THE NEW MODEL:</t>
+          <t>WHY OFFICE IS IMPUTED:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Office/bookings-team channel goes away. Those customers either self-serve online (→ shifts into revenue channel)</t>
+          <t xml:space="preserve">  Office bookings in the DMN xlsx show £0 price — they're placeholder reservations; payment settles at the venue till.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    or contact the venue directly (venue handles, no Holding Co involvement).</t>
+          <t xml:space="preserve">  We impute revenue as qty × SKU list price to show the real £ value of that channel. Swap in actual till takings</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Holding Co revenue = Booking Fee (10% on top) + Commission % (from venue gross). Online channel only.</t>
+          <t xml:space="preserve">  when available — the office team may comp/discount, in which case actual &lt; imputed.</t>
         </is>
       </c>
     </row>
@@ -586,73 +586,104 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>STRUCTURAL ASSUMPTIONS (v1):</t>
+          <t>UNDER THE NEW MODEL:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Booking fee: 10% added ON TOP of ticket at checkout. Kept by Holding Co. Funds online funnel.</t>
+          <t xml:space="preserve">  • Office/bookings-team channel goes away. Customers self-serve online (→ shifts into online channel, Holding Co</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Commission: SEPARATE % taken from VENUE on gross ticket sales. Holding Co's per-venue licensing fee.</t>
+          <t xml:space="preserve">    takes commission) or contact the venue directly (venue handles, no Holding Co).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Token value: £0.325 per arcade token, NO VAT. Each 'Golf + 4 Tokens' SKU bundles 4 tokens (£1.30/ticket).</t>
+          <t xml:space="preserve">  • Holding Co revenue = Booking Fee (10% on top of online ticket) + Commission % (from online venue gross).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Under new model tokens move to in-store TILL only — online SKUs will be re-priced to strip the token component.</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>STRUCTURAL ASSUMPTIONS (v1):</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>SHEETS:</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Booking fee: 10% added ON TOP of ticket at checkout. Kept by Holding Co. Online only.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Online SKUs 2025 — all online-portal tickets by SKU with token/booking-fee/revenue columns.</t>
+          <t xml:space="preserve">  • Commission: SEPARATE % taken from VENUE on gross online ticket sales.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Office SKUs 2025 — same structure for external/till bookings (revenue = £0 by system design).</t>
+          <t xml:space="preserve">  • Token value: £0.325 per arcade token, NO VAT. Each 'Golf + 4 Tokens' SKU bundles 4 tokens (£1.30/ticket).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Monthly 2025 — per-month online and office splits.</t>
+          <t xml:space="preserve">  • Under new model tokens move to in-store TILL only — online SKUs will be re-priced to strip the token component.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Model — interactive inputs (column B) driving Holding Co P&amp;L and venue net.</t>
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>SHEETS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Online SKUs 2025 — actual portal revenue per SKU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Office SKUs 2025 — imputed revenue per SKU (qty × list price). Booking Fee column = £0 (till sales don't carry it).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Monthly 2025 — per-month split + combined total revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Model — interactive inputs driving Holding Co P&amp;L and venue net (online only).</t>
         </is>
       </c>
     </row>
@@ -678,8 +709,8 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -690,7 +721,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="38" customHeight="1">
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>SKU</t>
@@ -737,7 +768,7 @@
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Gross Revenue 2025</t>
+          <t>Revenue 2025</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -1171,19 +1202,19 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>SECTION B · OFFICE / EXTERNAL BOOKINGS (Status = external) — Borough 2025 · Revenue £0 (settled at venue till)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="38" customHeight="1">
+          <t>SECTION B · OFFICE / EXTERNAL BOOKINGS (Status = external) — Borough 2025 · Revenue imputed at SKU list price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>SKU</t>
@@ -1230,12 +1261,14 @@
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Gross Revenue 2025</t>
+          <t>Revenue 2025
+(imputed at list price)</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Booking Fees 2025</t>
+          <t>Booking Fees 2025
+(n/a for till sales)</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -1272,7 +1305,7 @@
         <v>1977</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>0</v>
+        <v>31632</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>0</v>
@@ -1309,7 +1342,7 @@
         <v>1868</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0</v>
+        <v>23350</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>0</v>
@@ -1346,7 +1379,7 @@
         <v>268</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>0</v>
+        <v>2680</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>0</v>
@@ -1383,7 +1416,7 @@
         <v>8</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>0</v>
@@ -1420,7 +1453,7 @@
         <v>276</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0</v>
+        <v>3312</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>0</v>
@@ -1457,7 +1490,7 @@
         <v>12</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>0</v>
@@ -1494,7 +1527,7 @@
         <v>103</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0</v>
+        <v>515</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>0</v>
@@ -1630,7 +1663,7 @@
         <v>4512</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>0</v>
+        <v>61629</v>
       </c>
       <c r="J13" s="11" t="n">
         <v>0</v>
@@ -1653,7 +1686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1661,16 +1694,17 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>MONTHLY CHANNEL SPLIT — Borough 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>MONTHLY CHANNEL SPLIT — Borough 2025 (online actual · office imputed at list price)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Month</t>
@@ -1693,7 +1727,13 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Office Revenue</t>
+          <t>Office Revenue
+(imputed)</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1753,10 @@
         <v>298</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>0</v>
+        <v>3836.5</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>23425.8</v>
       </c>
     </row>
     <row r="4">
@@ -1732,7 +1775,10 @@
         <v>183</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0</v>
+        <v>2406.5</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>24433.2</v>
       </c>
     </row>
     <row r="5">
@@ -1751,7 +1797,10 @@
         <v>349</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0</v>
+        <v>4822</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>22195.2</v>
       </c>
     </row>
     <row r="6">
@@ -1770,7 +1819,10 @@
         <v>353</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0</v>
+        <v>4777.5</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>19993.3</v>
       </c>
     </row>
     <row r="7">
@@ -1789,7 +1841,10 @@
         <v>295</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0</v>
+        <v>4071.5</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>19427</v>
       </c>
     </row>
     <row r="8">
@@ -1808,7 +1863,10 @@
         <v>391</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0</v>
+        <v>5440.5</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>18089.2</v>
       </c>
     </row>
     <row r="9">
@@ -1827,7 +1885,10 @@
         <v>423</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0</v>
+        <v>5845.5</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>20344.3</v>
       </c>
     </row>
     <row r="10">
@@ -1846,7 +1907,10 @@
         <v>167</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0</v>
+        <v>2005.5</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>20650.45</v>
       </c>
     </row>
     <row r="11">
@@ -1865,7 +1929,10 @@
         <v>351</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0</v>
+        <v>5085.5</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>20213.2</v>
       </c>
     </row>
     <row r="12">
@@ -1884,7 +1951,10 @@
         <v>274</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0</v>
+        <v>4007.5</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>24786.5</v>
       </c>
     </row>
     <row r="13">
@@ -1903,7 +1973,10 @@
         <v>470</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0</v>
+        <v>6560</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>24988.25</v>
       </c>
     </row>
     <row r="14">
@@ -1922,7 +1995,10 @@
         <v>958</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0</v>
+        <v>12770.5</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>34246.3</v>
       </c>
     </row>
     <row r="15">
@@ -1941,12 +2017,15 @@
         <v>4512</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>0</v>
+        <v>61629</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>272792.7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 1.5pct payment processing fee; rename Holding Co to Plonk Golf
Payment fee (1.5pct) applied to all revenue that flows through the
online payment provider — online portal sales always, office bookings
whenever Plonk Golf processes them digitally via the bookings manager.
Sits as a cost line in the Plonk Golf P&L. At defaults this is roughly
£4,092 per year on £272,793 combined gross.

Renamed every Holding Co reference to Plonk Golf across the codebase:
- 7 in src/data.js
- 41 in src/tabs/IPLicensing.jsx
- 2 in src/tabs/Plonk.jsx (eyebrow label)
- 6 in src/tabs/PlonkCover.jsx (hero, copy)
- 2 in src/slides/FinancialPerformance.jsx (2025 cost note)
- 2 in CLAUDE.md
- Regenerated workbook/ip_licensing_2025.xlsx with PLONK GOLF headers
  plus the new payment-fee input + output rows in the Model sheet

JS identifiers also renamed (holdingCoRevenue/Costs/Net -> plonkGolf*).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/ip_licensing_2025.xlsx
+++ b/workbook/ip_licensing_2025.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IP &amp; LICENSING — BOROUGH 2025 (split by channel, all revenue coded in)</t>
+          <t>IP &amp; LICENSING — BOROUGH 2025 (split by channel, Plonk Golf × Venue)</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • OFFICE (Status = external):    4,512 tickets  £  61,629.00  ← IMPUTED at SKU list price (qty × price)</t>
+          <t xml:space="preserve">  • OFFICE (Status = external):    4,512 tickets  £  61,629.00  ← imputed at SKU list price</t>
         </is>
       </c>
     </row>
@@ -555,28 +555,28 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>WHY OFFICE IS IMPUTED:</t>
+          <t>UNDER THE NEW MODEL:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Office bookings in the DMN xlsx show £0 price — they're placeholder reservations; payment settles at the venue till.</t>
+          <t xml:space="preserve">  • Plonk Golf licenses the IP + runs the digital funnel. Revenue comes from booking fees + per-venue commission.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  We impute revenue as qty × SKU list price to show the real £ value of that channel. Swap in actual till takings</t>
+          <t xml:space="preserve">  • Office/bookings-team channel goes away unless Plonk Golf provides a bookings manager (conditional scenario).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  when available — the office team may comp/discount, in which case actual &lt; imputed.</t>
+          <t xml:space="preserve">  • Plonk Golf revenue = Booking Fee (10% on top) + Commission % × golf (online) + Commission % × golf (office, conditional).</t>
         </is>
       </c>
     </row>
@@ -586,104 +586,66 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>UNDER THE NEW MODEL:</t>
+          <t>STRUCTURAL ASSUMPTIONS (v1):</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Office/bookings-team channel goes away. Customers self-serve online (→ shifts into online channel, Holding Co</t>
+          <t xml:space="preserve">  • Booking fee: 10% added ON TOP of ticket at checkout. Customer-facing. Kept by Plonk Golf.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    takes commission) or contact the venue directly (venue handles, no Holding Co).</t>
+          <t xml:space="preserve">  • Commission: SEPARATE % taken from VENUE on gross golf ticket sales. Plonk Golf's per-venue licensing fee.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Holding Co revenue = Booking Fee (10% on top of online ticket) + Commission % (from online venue gross).</t>
+          <t xml:space="preserve">  • Payment processing: 1.5% on all online-processed revenue (online + office if digitally processed). Plonk Golf cost.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Token value: £0.325 per arcade token, NO VAT. Each 'Golf + 4 Tokens' SKU bundles 4 tokens (£1.30/ticket).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>STRUCTURAL ASSUMPTIONS (v1):</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Under new model tokens move to in-store TILL only — online SKUs will be re-priced to strip the token component.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Booking fee: 10% added ON TOP of ticket at checkout. Kept by Holding Co. Online only.</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Commission: SEPARATE % taken from VENUE on gross online ticket sales.</t>
+          <t>NOTE: The Model sheet shows commission × GROSS (100% golf share). In the React UI, commission is scoped to golf-only SKUs</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Token value: £0.325 per arcade token, NO VAT. Each 'Golf + 4 Tokens' SKU bundles 4 tokens (£1.30/ticket).</t>
+          <t xml:space="preserve">  (excluding pool tables, pool tournament, extra tokens and Valentine's Day). Golf share ≈ 97% of gross — re-model in Excel</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Under new model tokens move to in-store TILL only — online SKUs will be re-priced to strip the token component.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>SHEETS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Online SKUs 2025 — actual portal revenue per SKU.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Office SKUs 2025 — imputed revenue per SKU (qty × list price). Booking Fee column = £0 (till sales don't carry it).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Monthly 2025 — per-month split + combined total revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Model — interactive inputs driving Holding Co P&amp;L and venue net (online only).</t>
+          <t xml:space="preserve">  with an explicit golf-share input if/when you need higher precision.</t>
         </is>
       </c>
     </row>
@@ -2037,18 +1999,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HOLDING CO × VENUE — COMMISSION MODEL (online only)</t>
+          <t>PLONK GOLF × VENUE — COMMISSION MODEL</t>
         </is>
       </c>
     </row>
@@ -2077,37 +2039,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Volume uplift %</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="n">
-        <v>0</v>
+          <t>Gross office sales baseline (imputed 2025)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>61629</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>test scenarios</t>
+          <t>from Office SKUs sheet</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Commission % (from venue)</t>
+          <t>Volume uplift %</t>
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>slider default 10%</t>
+          <t>test scenarios</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Booking fee % (on top, customer pays)</t>
+          <t>Commission % — online golf</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
@@ -2115,162 +2077,284 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>locked — online funnel cost</t>
+          <t>slider default 10%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Maintenance (12 × £250)</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>3000</v>
+          <t>Commission % — office golf (bookings manager)</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>0.1</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>conditional scenario</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Website + booking system</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>6000</v>
+          <t>Booking fee % (on top, customer pays)</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>0.1</v>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>locked — online funnel cost</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SEO (non-venue-specific)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>6000</v>
+          <t>Payment processing % (Stripe or similar)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>0.015</v>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>Plonk Golf cost on all online-processed revenue</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Chatbot / AI booking</t>
+          <t>Maintenance (12 × £250)</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>1200</v>
+        <v>3000</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
+          <t>fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Website + booking system</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
           <t>slider</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>OUTPUTS</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SEO (non-venue-specific)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>slider</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gross online sales (adjusted)</t>
-        </is>
-      </c>
-      <c r="B14" s="6">
-        <f>B4*(1+B5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Booking fees collected</t>
-        </is>
-      </c>
-      <c r="B15" s="6">
-        <f>B14*B7</f>
-        <v/>
+          <t>Chatbot / AI booking</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Commission from venue</t>
-        </is>
-      </c>
-      <c r="B16" s="6">
-        <f>B14*B6</f>
-        <v/>
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>OUTPUTS</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Holding Co revenue</t>
+          <t>Gross online sales (adjusted)</t>
         </is>
       </c>
       <c r="B17" s="6">
-        <f>B15+B16</f>
+        <f>B4*(1+B6)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Total Holding Co costs</t>
+          <t>Gross office sales (adjusted)</t>
         </is>
       </c>
       <c r="B18" s="6">
-        <f>B8+B9+B10+B11</f>
+        <f>B5*(1+B6)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NET to Holding Co</t>
+          <t>Booking fees collected (online × 10%)</t>
         </is>
       </c>
       <c r="B19" s="6">
-        <f>B17-B18</f>
+        <f>B17*B9</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Token cost (venue COGS)</t>
+          <t>Commission from Venue — Online (× golf share assumed 100%)</t>
         </is>
       </c>
       <c r="B20" s="6">
-        <f>(1+B5)*17612.4</f>
+        <f>B17*B7</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Commission from Venue — Office (× golf share assumed 100%)</t>
+        </is>
+      </c>
+      <c r="B21" s="6">
+        <f>B18*B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Plonk Golf revenue</t>
+        </is>
+      </c>
+      <c r="B22" s="6">
+        <f>B19+B20+B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>− Payment processing (1.5% × online + office)</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
+        <f>(B17+B18)*B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>− Maintenance (12 × £250)</t>
+        </is>
+      </c>
+      <c r="B24" s="6">
+        <f>B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>− Website + booking system</t>
+        </is>
+      </c>
+      <c r="B25" s="6">
+        <f>B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>− SEO</t>
+        </is>
+      </c>
+      <c r="B26" s="6">
+        <f>B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>− Chatbot / AI booking</t>
+        </is>
+      </c>
+      <c r="B27" s="6">
+        <f>B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Total Plonk Golf costs</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>B23+B24+B25+B26+B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>NET to Plonk Golf</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>B22-B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Token cost (venue COGS)</t>
+        </is>
+      </c>
+      <c r="B30" s="6">
+        <f>(1+B6)*17612.4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>NET to venue (online)</t>
         </is>
       </c>
-      <c r="B21" s="6">
-        <f>B14-B16-B20</f>
+      <c r="B31" s="6">
+        <f>B17-B20-B30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
IP & Licensing: add Accountancy fees (£3k/yr) to Plonk Golf costs
New slider in the Plonk Golf × Venue model (default £3,000/yr, range
0–£15k, step £250). Feeds into the Plonk Golf P&L as a new cost line
between "Chatbot / AI booking" and "Payment processing".

xlsx Model sheet regenerated: new input row for Accountancy fees at
B15, cost formula updated to include it, README lists the full 2026
baseline cost stack for reference.

At defaults, total Plonk Golf costs rise from £20,292 to £23,292.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/ip_licensing_2025.xlsx
+++ b/workbook/ip_licensing_2025.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -586,64 +586,116 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>STRUCTURAL ASSUMPTIONS (v1):</t>
+          <t>PLONK GOLF COSTS (2026 baseline):</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Booking fee: 10% added ON TOP of ticket at checkout. Customer-facing. Kept by Plonk Golf.</t>
+          <t xml:space="preserve">  • Maintenance (fixed):        £3,000/yr (12 × £250)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Commission: SEPARATE % taken from VENUE on gross golf ticket sales. Plonk Golf's per-venue licensing fee.</t>
+          <t xml:space="preserve">  • Website + booking system:   £6,000/yr</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Payment processing: 1.5% on all online-processed revenue (online + office if digitally processed). Plonk Golf cost.</t>
+          <t xml:space="preserve">  • SEO (non-venue-specific):   £6,000/yr</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Token value: £0.325 per arcade token, NO VAT. Each 'Golf + 4 Tokens' SKU bundles 4 tokens (£1.30/ticket).</t>
+          <t xml:space="preserve">  • Chatbot / AI booking:       £1,200/yr</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Under new model tokens move to in-store TILL only — online SKUs will be re-priced to strip the token component.</t>
+          <t xml:space="preserve">  • Accountancy fees:           £3,000/yr</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Payment processing:         1.5% × (online + office gross)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>NOTE: The Model sheet shows commission × GROSS (100% golf share). In the React UI, commission is scoped to golf-only SKUs</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (excluding pool tables, pool tournament, extra tokens and Valentine's Day). Golf share ≈ 97% of gross — re-model in Excel</t>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>STRUCTURAL ASSUMPTIONS (v1):</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Booking fee: 10% added ON TOP of ticket at checkout. Customer-facing. Kept by Plonk Golf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Commission: SEPARATE % taken from VENUE on gross golf ticket sales. Plonk Golf's per-venue licensing fee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Payment processing: 1.5% on all online-processed revenue (online + office if digitally processed). Plonk Golf cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Token value: £0.325 per arcade token, NO VAT. Each 'Golf + 4 Tokens' SKU bundles 4 tokens (£1.30/ticket).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Under new model tokens move to in-store TILL only — online SKUs will be re-priced to strip the token component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>NOTE: The Model sheet shows commission × GROSS (100% golf share). In the React UI, commission is scoped to golf-only SKUs</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (excluding pool tables, pool tournament, extra tokens and Valentine's Day). Golf share ≈ 97% of gross — re-model in Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  with an explicit golf-share input if/when you need higher precision.</t>
         </is>
@@ -1999,7 +2051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2186,175 +2238,201 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Accountancy fees</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>slider default £3k/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>OUTPUTS</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Gross online sales (adjusted)</t>
         </is>
       </c>
-      <c r="B17" s="6">
+      <c r="B18" s="6">
         <f>B4*(1+B6)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Gross office sales (adjusted)</t>
         </is>
       </c>
-      <c r="B18" s="6">
+      <c r="B19" s="6">
         <f>B5*(1+B6)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Booking fees collected (online × 10%)</t>
-        </is>
-      </c>
-      <c r="B19" s="6">
-        <f>B17*B9</f>
-        <v/>
-      </c>
-    </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Commission from Venue — Online (× golf share assumed 100%)</t>
+          <t>Booking fees collected (online × 10%)</t>
         </is>
       </c>
       <c r="B20" s="6">
-        <f>B17*B7</f>
+        <f>B18*B9</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Commission from Venue — Office (× golf share assumed 100%)</t>
+          <t>Commission from Venue — Online (× golf share assumed 100%)</t>
         </is>
       </c>
       <c r="B21" s="6">
-        <f>B18*B8</f>
+        <f>B18*B7</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Plonk Golf revenue</t>
+          <t>Commission from Venue — Office (× golf share assumed 100%)</t>
         </is>
       </c>
       <c r="B22" s="6">
-        <f>B19+B20+B21</f>
+        <f>B19*B8</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>− Payment processing (1.5% × online + office)</t>
+          <t>Plonk Golf revenue</t>
         </is>
       </c>
       <c r="B23" s="6">
-        <f>(B17+B18)*B10</f>
+        <f>B20+B21+B22</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>− Payment processing (1.5% × online + office)</t>
+        </is>
+      </c>
+      <c r="B24" s="6">
+        <f>(B18+B19)*B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>− Maintenance (12 × £250)</t>
         </is>
       </c>
-      <c r="B24" s="6">
+      <c r="B25" s="6">
         <f>B11</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>− Website + booking system</t>
         </is>
       </c>
-      <c r="B25" s="6">
+      <c r="B26" s="6">
         <f>B12</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>− SEO</t>
         </is>
       </c>
-      <c r="B26" s="6">
+      <c r="B27" s="6">
         <f>B13</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>− Chatbot / AI booking</t>
         </is>
       </c>
-      <c r="B27" s="6">
+      <c r="B28" s="6">
         <f>B14</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Total Plonk Golf costs</t>
-        </is>
-      </c>
-      <c r="B28" s="6">
-        <f>B23+B24+B25+B26+B27</f>
-        <v/>
-      </c>
-    </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NET to Plonk Golf</t>
+          <t>− Accountancy fees</t>
         </is>
       </c>
       <c r="B29" s="6">
-        <f>B22-B28</f>
+        <f>B15</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Total Plonk Golf costs</t>
+        </is>
+      </c>
+      <c r="B30" s="6">
+        <f>B24+B25+B26+B27+B28+B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>NET to Plonk Golf</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>B23-B30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Token cost (venue COGS)</t>
         </is>
       </c>
-      <c r="B30" s="6">
+      <c r="B32" s="6">
         <f>(1+B6)*17612.4</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>NET to venue (online)</t>
         </is>
       </c>
-      <c r="B31" s="6">
-        <f>B17-B20-B30</f>
+      <c r="B33" s="6">
+        <f>B18-B21-B32</f>
         <v/>
       </c>
     </row>

</xml_diff>